<commit_message>
content: update airbrush application info in product-info.xlsx
</commit_message>
<xml_diff>
--- a/docs/product-info.xlsx
+++ b/docs/product-info.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BFB2189-BD85-42C5-AA1D-84324160A0EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{870D6F65-3967-44D3-A191-D5190FFE9294}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="606" uniqueCount="213">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="668" uniqueCount="234">
   <si>
     <t>key</t>
   </si>
@@ -699,79 +699,70 @@
     <t>EQUIPMENT::AIR BRUSH</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Introduction to the World of Airbrushing
-What is an airbrush?
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">An airbrush is a small spray gun that applies colour in a controlled way using compressed air.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">The main parts of an airbrush are:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Pen
-Colour cup
-Needle
-Nozzle
-Spray tip
-Needle seal — Teflon
-Base unit
-The required amount of colour is placed into the colour cup. The needle completely closes the nozzle when the airbrush is not in use. When the airbrush is activated, the compressed air starts and the needle slowly pulls back from the nozzle, opening a small gap around the needle so the colour can be sprayed through the nozzle by the compressed air.
-The needle helps create detailed work, as the cone at the tip of the needle guides the colour particles to the tip. This provides excellent detail with smooth and even coverage on small surfaces, such as nails.
-Airbrushes have needle and head seals made from Teflon™ or rubber. Seals made from Teflon™ are resistant to almost all materials that can be sprayed with an airbrush. This means that solvent-based colours or other stronger materials can be sprayed without any issue.
-What can I do with an airbrush?
-An airbrush is the ideal tool for applying fine colour particles to all kinds of surfaces. This means you can decorate or customise many different objects with an airbrush.
-Some examples include:
-Custom colour decoration of devices or objects, such as phone cases, helmets, clothing, surfboards, etc.
-Painting model ships, airplanes, cars, dioramas, etc.
-Application on figures, dolls, etc.
-Custom painting of real cars, motorcycles, trucks, etc.
-Repairing small paint damage on real cars, motorcycles, boats, airplanes, etc.
-Dental laboratories, for matching the colour of white porcelain teeth to the patient’s natural tooth colour.
-Applying food colouring to biscuits, cakes, pastries, etc.
-Weathering techniques on models, such as rust and mud effects on model trains, cars, etc.
-Airbrush colours
-The colours used in nail airbrushing are acrylic colours and specially diluted semi-permanent gel colours.
-Acrylic colour has one major disadvantage for the nail technician: the so-called drying effect. When the nozzle is not large enough for the colour to flow properly, the air passing through can dry the colour. As a result, more time is spent cleaning the airbrush than actually spraying.
-With the specially diluted GEL.IT.UP colours, this effect is reduced, allowing for faster colour changes and easier, quicker cleaning.
-Cleaning the airbrush
-The airbrush should be cleaned with a special airbrush cleaner or with our well-known cleanser.
-At the end of the day, after all appointments are completed, the airbrush should be cleaned thoroughly and in detail, including removing and cleaning the needle.</t>
-    </r>
+    <t>Introduction to the World of Airbrushing What is an airbrush? An airbrush is a small spray gun that applies colour in a controlled way using compressed air.</t>
+  </si>
+  <si>
+    <t>The main parts of an airbrush are:</t>
+  </si>
+  <si>
+    <t>Pen</t>
+  </si>
+  <si>
+    <t>Colour Cup</t>
+  </si>
+  <si>
+    <t>Needle</t>
+  </si>
+  <si>
+    <t>Nozzle</t>
+  </si>
+  <si>
+    <t>Spray Tip</t>
+  </si>
+  <si>
+    <t>Needle Seal</t>
+  </si>
+  <si>
+    <t>Base Unit</t>
+  </si>
+  <si>
+    <t>Application - Acrylic colour has one major disadvantage for nail technicians: the drying effect.</t>
+  </si>
+  <si>
+    <t>Application - When the nozzle is not large enough for the colour to flow correctly, the passing air can dry the colour.</t>
+  </si>
+  <si>
+    <t>Application - This can result in spending more time cleaning the airbrush than actually spraying.</t>
+  </si>
+  <si>
+    <t>Application - Specially diluted GEL.IT.UP colours reduce this issue.</t>
+  </si>
+  <si>
+    <t>These allow for Faster colour changes, easier cleaning and quicker workflow</t>
+  </si>
+  <si>
+    <t>Airbrush Colours:  Acrylic Colours or Specially diluted semi-permanent gel colours</t>
+  </si>
+  <si>
+    <t>Cleaning your Airbrush</t>
+  </si>
+  <si>
+    <t>Cleaning - The airbrush should be cleaned with:  Special airbrush cleaner or All-in-One Liqiud</t>
+  </si>
+  <si>
+    <t>Cleaning - At the end of the working day, after all appointments are completed:</t>
+  </si>
+  <si>
+    <t>Cleaning - Clean the airbrush thoroughly.</t>
+  </si>
+  <si>
+    <t>Cleaning - Remove and clean the needle.</t>
+  </si>
+  <si>
+    <t>Cleaning - Make sure all product residue is removed.</t>
+  </si>
+  <si>
+    <t>Usage - Place the required amount of colour into the colour cup. When activated, compressed air pulls the needle back, allowing the colour to spray through the nozzle in a controlled flow.</t>
   </si>
 </sst>
 </file>
@@ -1246,7 +1237,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C203"/>
+  <dimension ref="A1:C224"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
@@ -3162,322 +3153,551 @@
         <v>110</v>
       </c>
     </row>
-    <row r="175" spans="1:3" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A175" s="10" t="s">
         <v>211</v>
       </c>
       <c r="B175" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="C175" s="3" t="s">
+      <c r="C175" s="1" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="176" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A176" s="7" t="s">
-        <v>111</v>
-      </c>
-      <c r="B176" s="8" t="s">
-        <v>4</v>
-      </c>
-      <c r="C176" s="9" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="177" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A177" s="7" t="s">
-        <v>111</v>
-      </c>
-      <c r="B177" s="8" t="s">
-        <v>4</v>
-      </c>
-      <c r="C177" s="9" t="s">
-        <v>113</v>
+    <row r="176" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A176" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="B176" s="12" t="s">
+        <v>4</v>
+      </c>
+      <c r="C176" s="1" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="177" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A177" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="B177" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="C177" s="3" t="s">
+        <v>214</v>
       </c>
     </row>
     <row r="178" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A178" s="7" t="s">
-        <v>111</v>
-      </c>
-      <c r="B178" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="C178" s="9" t="s">
-        <v>114</v>
+      <c r="A178" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="B178" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="C178" s="3" t="s">
+        <v>215</v>
       </c>
     </row>
     <row r="179" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A179" s="7" t="s">
-        <v>111</v>
-      </c>
-      <c r="B179" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="C179" s="9" t="s">
-        <v>115</v>
+      <c r="A179" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="B179" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="C179" s="3" t="s">
+        <v>216</v>
       </c>
     </row>
     <row r="180" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A180" s="7" t="s">
-        <v>204</v>
-      </c>
-      <c r="B180" s="13" t="s">
-        <v>4</v>
-      </c>
-      <c r="C180" s="4" t="s">
-        <v>209</v>
+      <c r="A180" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="B180" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="C180" s="3" t="s">
+        <v>217</v>
       </c>
     </row>
     <row r="181" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A181" s="7" t="s">
-        <v>204</v>
-      </c>
-      <c r="B181" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="C181" s="9" t="s">
-        <v>210</v>
+      <c r="A181" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="B181" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="C181" s="3" t="s">
+        <v>218</v>
       </c>
     </row>
     <row r="182" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A182" s="7" t="s">
-        <v>204</v>
-      </c>
-      <c r="B182" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="C182" s="9" t="s">
-        <v>205</v>
+      <c r="A182" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="B182" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="C182" s="3" t="s">
+        <v>219</v>
       </c>
     </row>
     <row r="183" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A183" s="7" t="s">
-        <v>204</v>
-      </c>
-      <c r="B183" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="C183" s="9" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="184" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A184" s="7" t="s">
-        <v>204</v>
-      </c>
-      <c r="B184" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="C184" s="9" t="s">
-        <v>207</v>
+      <c r="A183" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="B183" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="C183" s="3" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="184" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A184" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="B184" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="C184" s="3" t="s">
+        <v>233</v>
       </c>
     </row>
     <row r="185" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A185" s="7" t="s">
-        <v>204</v>
-      </c>
-      <c r="B185" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="C185" s="9" t="s">
-        <v>208</v>
+      <c r="A185" s="10"/>
+      <c r="B185" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="C185" s="3" t="s">
+        <v>226</v>
       </c>
     </row>
     <row r="186" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A186" s="10" t="s">
-        <v>116</v>
-      </c>
-      <c r="B186" s="11" t="s">
-        <v>4</v>
+        <v>211</v>
+      </c>
+      <c r="B186" s="12" t="s">
+        <v>10</v>
       </c>
       <c r="C186" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="187" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="187" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A187" s="10" t="s">
-        <v>116</v>
-      </c>
-      <c r="B187" s="11" t="s">
-        <v>4</v>
+        <v>211</v>
+      </c>
+      <c r="B187" s="12" t="s">
+        <v>10</v>
       </c>
       <c r="C187" s="3" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="188" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="188" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A188" s="10" t="s">
-        <v>116</v>
-      </c>
-      <c r="B188" s="11" t="s">
-        <v>4</v>
+        <v>211</v>
+      </c>
+      <c r="B188" s="12" t="s">
+        <v>10</v>
       </c>
       <c r="C188" s="3" t="s">
-        <v>118</v>
+        <v>223</v>
       </c>
     </row>
     <row r="189" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A189" s="7" t="s">
-        <v>119</v>
-      </c>
-      <c r="B189" s="8" t="s">
-        <v>4</v>
-      </c>
-      <c r="C189" s="9" t="s">
-        <v>120</v>
+      <c r="A189" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="B189" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="C189" s="3" t="s">
+        <v>224</v>
       </c>
     </row>
     <row r="190" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A190" s="7" t="s">
-        <v>119</v>
-      </c>
-      <c r="B190" s="8" t="s">
-        <v>4</v>
-      </c>
-      <c r="C190" s="9" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="191" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A190" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="B190" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="C190" s="3" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="191" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A191" s="10" t="s">
-        <v>122</v>
-      </c>
-      <c r="B191" s="11" t="s">
-        <v>4</v>
+        <v>211</v>
+      </c>
+      <c r="B191" s="12" t="s">
+        <v>10</v>
       </c>
       <c r="C191" s="3" t="s">
-        <v>123</v>
+        <v>227</v>
       </c>
     </row>
     <row r="192" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A192" s="10" t="s">
-        <v>122</v>
-      </c>
-      <c r="B192" s="11" t="s">
-        <v>4</v>
+        <v>211</v>
+      </c>
+      <c r="B192" s="12" t="s">
+        <v>10</v>
       </c>
       <c r="C192" s="3" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="193" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A193" s="7" t="s">
-        <v>125</v>
-      </c>
-      <c r="B193" s="8" t="s">
-        <v>4</v>
-      </c>
-      <c r="C193" s="9" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="194" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A194" s="7" t="s">
-        <v>125</v>
-      </c>
-      <c r="B194" s="8" t="s">
-        <v>4</v>
-      </c>
-      <c r="C194" s="9" t="s">
-        <v>127</v>
+        <v>228</v>
+      </c>
+    </row>
+    <row r="193" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A193" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="B193" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="C193" s="3" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="194" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A194" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="B194" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="C194" s="3" t="s">
+        <v>230</v>
       </c>
     </row>
     <row r="195" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A195" s="7" t="s">
-        <v>125</v>
-      </c>
-      <c r="B195" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="C195" s="9" t="s">
-        <v>128</v>
+      <c r="A195" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="B195" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="C195" s="3" t="s">
+        <v>231</v>
       </c>
     </row>
     <row r="196" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A196" s="7" t="s">
-        <v>125</v>
-      </c>
-      <c r="B196" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="C196" s="9" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="197" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A196" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="B196" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="C196" s="3" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="197" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A197" s="7" t="s">
-        <v>125</v>
-      </c>
-      <c r="B197" s="13" t="s">
-        <v>10</v>
+        <v>111</v>
+      </c>
+      <c r="B197" s="8" t="s">
+        <v>4</v>
       </c>
       <c r="C197" s="9" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="198" spans="1:3" x14ac:dyDescent="0.3">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="198" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A198" s="7" t="s">
-        <v>125</v>
-      </c>
-      <c r="B198" s="13" t="s">
-        <v>10</v>
+        <v>111</v>
+      </c>
+      <c r="B198" s="8" t="s">
+        <v>4</v>
       </c>
       <c r="C198" s="9" t="s">
-        <v>131</v>
+        <v>113</v>
       </c>
     </row>
     <row r="199" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A199" s="7" t="s">
-        <v>125</v>
+        <v>111</v>
       </c>
       <c r="B199" s="13" t="s">
         <v>10</v>
       </c>
       <c r="C199" s="9" t="s">
-        <v>132</v>
+        <v>114</v>
       </c>
     </row>
     <row r="200" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A200" s="7" t="s">
-        <v>125</v>
+        <v>111</v>
       </c>
       <c r="B200" s="13" t="s">
         <v>10</v>
       </c>
       <c r="C200" s="9" t="s">
-        <v>133</v>
+        <v>115</v>
       </c>
     </row>
     <row r="201" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A201" s="7" t="s">
-        <v>125</v>
+        <v>204</v>
       </c>
       <c r="B201" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="C201" s="9" t="s">
-        <v>134</v>
+        <v>4</v>
+      </c>
+      <c r="C201" s="4" t="s">
+        <v>209</v>
       </c>
     </row>
     <row r="202" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A202" s="7" t="s">
+        <v>204</v>
+      </c>
+      <c r="B202" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="C202" s="9" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="203" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A203" s="7" t="s">
+        <v>204</v>
+      </c>
+      <c r="B203" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="C203" s="9" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="204" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A204" s="7" t="s">
+        <v>204</v>
+      </c>
+      <c r="B204" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="C204" s="9" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="205" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A205" s="7" t="s">
+        <v>204</v>
+      </c>
+      <c r="B205" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="C205" s="9" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="206" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A206" s="7" t="s">
+        <v>204</v>
+      </c>
+      <c r="B206" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="C206" s="9" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="207" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A207" s="10" t="s">
+        <v>116</v>
+      </c>
+      <c r="B207" s="11" t="s">
+        <v>4</v>
+      </c>
+      <c r="C207" s="3" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="208" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A208" s="10" t="s">
+        <v>116</v>
+      </c>
+      <c r="B208" s="11" t="s">
+        <v>4</v>
+      </c>
+      <c r="C208" s="3" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="209" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A209" s="10" t="s">
+        <v>116</v>
+      </c>
+      <c r="B209" s="11" t="s">
+        <v>4</v>
+      </c>
+      <c r="C209" s="3" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="210" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A210" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="B210" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="C210" s="9" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="211" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A211" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="B211" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="C211" s="9" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="212" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A212" s="10" t="s">
+        <v>122</v>
+      </c>
+      <c r="B212" s="11" t="s">
+        <v>4</v>
+      </c>
+      <c r="C212" s="3" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="213" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A213" s="10" t="s">
+        <v>122</v>
+      </c>
+      <c r="B213" s="11" t="s">
+        <v>4</v>
+      </c>
+      <c r="C213" s="3" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="214" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A214" s="7" t="s">
         <v>125</v>
       </c>
-      <c r="B202" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="C202" s="9" t="s">
+      <c r="B214" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="C214" s="9" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="215" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A215" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="B215" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="C215" s="9" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="216" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A216" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="B216" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="C216" s="9" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="217" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A217" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="B217" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="C217" s="9" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="218" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A218" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="B218" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="C218" s="9" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="219" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A219" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="B219" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="C219" s="9" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="220" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A220" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="B220" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="C220" s="9" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="221" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A221" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="B221" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="C221" s="9" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="222" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A222" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="B222" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="C222" s="9" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="223" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A223" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="B223" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="C223" s="9" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="203" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A203" s="10" t="s">
+    <row r="224" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A224" s="10" t="s">
         <v>136</v>
       </c>
-      <c r="B203" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="C203" s="3" t="s">
+      <c r="B224" s="11" t="s">
+        <v>4</v>
+      </c>
+      <c r="C224" s="3" t="s">
         <v>173</v>
       </c>
     </row>

</xml_diff>